<commit_message>
Updated 'Gear Study Summary' table logic to correctly compute exact site-visit intersections for independent sample counts.
</commit_message>
<xml_diff>
--- a/output/tables/AICTables_GLMM.xlsx
+++ b/output/tables/AICTables_GLMM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ostatemailokstate-my.sharepoint.com/personal/tanner_scholten_okstate_edu/Documents/Thesis Project/Data/R/output/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_191CD68A036A66B0DFE9CE2EC4B9B4912D76B7AF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D4948C8-66CA-4B92-8E94-18D3AECE4C37}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_191CD68A036A66B0DFE9CE2EC4B9B4912D76B7AF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1DE7ADD-25E0-4408-8278-C56019F46F83}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ModelList" sheetId="1" r:id="rId1"/>
@@ -3129,6 +3129,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.6328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -3320,22 +3330,22 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D8" s="1">
-        <v>-0.19209833496929299</v>
+        <v>1.9336499784206</v>
       </c>
       <c r="E8" s="1">
-        <v>0.16056978757113199</v>
+        <v>0.224291665416988</v>
       </c>
       <c r="F8" s="1">
-        <v>-0.50681511860871098</v>
+        <v>1.49403831420331</v>
       </c>
       <c r="G8" s="1">
-        <v>0.122618448670125</v>
+        <v>2.3732616426379001</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -3346,19 +3356,19 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D9" s="1">
-        <v>0.12940878972786801</v>
+        <v>-0.19209833496929299</v>
       </c>
       <c r="E9" s="1">
-        <v>0.180169780953022</v>
+        <v>0.16056978757113199</v>
       </c>
       <c r="F9" s="1">
-        <v>-0.223723980940055</v>
+        <v>-0.50681511860871098</v>
       </c>
       <c r="G9" s="1">
-        <v>0.48254156039579099</v>
+        <v>0.122618448670125</v>
       </c>
       <c r="H9" t="s">
         <v>72</v>
@@ -3372,22 +3382,22 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D10" s="1">
-        <v>0.25501042332364898</v>
+        <v>0.12940878972786801</v>
       </c>
       <c r="E10" s="1">
-        <v>9.7520812074004704E-2</v>
+        <v>0.180169780953022</v>
       </c>
       <c r="F10" s="1">
-        <v>6.3869631658599393E-2</v>
+        <v>-0.223723980940055</v>
       </c>
       <c r="G10" s="1">
-        <v>0.44615121498869798</v>
+        <v>0.48254156039579099</v>
       </c>
       <c r="H10" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -3398,19 +3408,19 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D11" s="1">
-        <v>-0.50480848353284102</v>
+        <v>0.25501042332364898</v>
       </c>
       <c r="E11" s="1">
-        <v>0.20329704982144101</v>
+        <v>9.7520812074004704E-2</v>
       </c>
       <c r="F11" s="1">
-        <v>-0.90327070118286501</v>
+        <v>6.3869631658599393E-2</v>
       </c>
       <c r="G11" s="1">
-        <v>-0.106346265882816</v>
+        <v>0.44615121498869798</v>
       </c>
       <c r="H11" t="s">
         <v>127</v>
@@ -3424,19 +3434,19 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D12" s="1">
-        <v>1.9336499784206</v>
+        <v>-0.50480848353284102</v>
       </c>
       <c r="E12" s="1">
-        <v>0.224291665416988</v>
+        <v>0.20329704982144101</v>
       </c>
       <c r="F12" s="1">
-        <v>1.49403831420331</v>
+        <v>-0.90327070118286501</v>
       </c>
       <c r="G12" s="1">
-        <v>2.3732616426379001</v>
+        <v>-0.106346265882816</v>
       </c>
       <c r="H12" t="s">
         <v>127</v>
@@ -3554,19 +3564,19 @@
         <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D17" s="1">
-        <v>-0.111475850682123</v>
+        <v>0.37986242272303999</v>
       </c>
       <c r="E17" s="1">
-        <v>5.2574692982259898E-2</v>
+        <v>0.129990776757541</v>
       </c>
       <c r="F17" s="1">
-        <v>-0.214522248927352</v>
+        <v>0.12508050027826001</v>
       </c>
       <c r="G17" s="1">
-        <v>-8.4294524368934108E-3</v>
+        <v>0.63464434516781998</v>
       </c>
       <c r="H17" t="s">
         <v>127</v>
@@ -3580,22 +3590,22 @@
         <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D18" s="1">
-        <v>-8.9562595313452897E-2</v>
+        <v>-0.111475850682123</v>
       </c>
       <c r="E18" s="1">
-        <v>9.6549943038695699E-2</v>
+        <v>5.2574692982259898E-2</v>
       </c>
       <c r="F18" s="1">
-        <v>-0.278800483669296</v>
+        <v>-0.214522248927352</v>
       </c>
       <c r="G18" s="1">
-        <v>9.9675293042390603E-2</v>
+        <v>-8.4294524368934108E-3</v>
       </c>
       <c r="H18" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -3606,22 +3616,22 @@
         <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D19" s="1">
-        <v>-0.31532806917905998</v>
+        <v>-8.9562595313452897E-2</v>
       </c>
       <c r="E19" s="1">
-        <v>0.158759242897934</v>
+        <v>9.6549943038695699E-2</v>
       </c>
       <c r="F19" s="1">
-        <v>-0.62649618525901096</v>
+        <v>-0.278800483669296</v>
       </c>
       <c r="G19" s="1">
-        <v>-4.1599530991096E-3</v>
+        <v>9.9675293042390603E-2</v>
       </c>
       <c r="H19" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
@@ -3632,22 +3642,22 @@
         <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D20" s="1">
-        <v>-0.104959559484556</v>
+        <v>-0.31532806917905998</v>
       </c>
       <c r="E20" s="1">
-        <v>6.0271958236356601E-2</v>
+        <v>0.158759242897934</v>
       </c>
       <c r="F20" s="1">
-        <v>-0.223092597627815</v>
+        <v>-0.62649618525901096</v>
       </c>
       <c r="G20" s="1">
-        <v>1.3173478658703001E-2</v>
+        <v>-4.1599530991096E-3</v>
       </c>
       <c r="H20" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -3658,22 +3668,22 @@
         <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D21" s="1">
-        <v>-0.22511782150923601</v>
+        <v>-0.104959559484556</v>
       </c>
       <c r="E21" s="1">
-        <v>0.11397019754303001</v>
+        <v>6.0271958236356601E-2</v>
       </c>
       <c r="F21" s="1">
-        <v>-0.44849940869357402</v>
+        <v>-0.223092597627815</v>
       </c>
       <c r="G21" s="1">
-        <v>-1.73623432489678E-3</v>
+        <v>1.3173478658703001E-2</v>
       </c>
       <c r="H21" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -3684,22 +3694,22 @@
         <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D22" s="1">
-        <v>-0.157320927740038</v>
+        <v>-0.22511782150923601</v>
       </c>
       <c r="E22" s="1">
-        <v>8.9718215298701207E-2</v>
+        <v>0.11397019754303001</v>
       </c>
       <c r="F22" s="1">
-        <v>-0.33316862972549199</v>
+        <v>-0.44849940869357402</v>
       </c>
       <c r="G22" s="1">
-        <v>1.8526774245416499E-2</v>
+        <v>-1.73623432489678E-3</v>
       </c>
       <c r="H22" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
@@ -3710,22 +3720,22 @@
         <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D23" s="1">
-        <v>0.37986242272303999</v>
+        <v>-0.157320927740038</v>
       </c>
       <c r="E23" s="1">
-        <v>0.129990776757541</v>
+        <v>8.9718215298701207E-2</v>
       </c>
       <c r="F23" s="1">
-        <v>0.12508050027826001</v>
+        <v>-0.33316862972549199</v>
       </c>
       <c r="G23" s="1">
-        <v>0.63464434516781998</v>
+        <v>1.8526774245416499E-2</v>
       </c>
       <c r="H23" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
@@ -3736,19 +3746,19 @@
         <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D24" s="1">
-        <v>-0.47627518629238003</v>
+        <v>-0.29049982933698298</v>
       </c>
       <c r="E24" s="1">
-        <v>0.15106918820284801</v>
+        <v>0.147950730600625</v>
       </c>
       <c r="F24" s="1">
-        <v>-0.77237079516996299</v>
+        <v>-0.58048326131420802</v>
       </c>
       <c r="G24" s="1">
-        <v>-0.18017957741479701</v>
+        <v>-5.1639735975728097E-4</v>
       </c>
       <c r="H24" t="s">
         <v>127</v>
@@ -3762,19 +3772,19 @@
         <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D25" s="1">
-        <v>-0.29049982933698298</v>
+        <v>-0.47627518629238003</v>
       </c>
       <c r="E25" s="1">
-        <v>0.147950730600625</v>
+        <v>0.15106918820284801</v>
       </c>
       <c r="F25" s="1">
-        <v>-0.58048326131420802</v>
+        <v>-0.77237079516996299</v>
       </c>
       <c r="G25" s="1">
-        <v>-5.1639735975728097E-4</v>
+        <v>-0.18017957741479701</v>
       </c>
       <c r="H25" t="s">
         <v>127</v>
@@ -3840,22 +3850,22 @@
         <v>69</v>
       </c>
       <c r="C28" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D28" s="1">
-        <v>-0.15848678756562401</v>
+        <v>4.5963112216243399E-2</v>
       </c>
       <c r="E28" s="1">
-        <v>4.6517045756649403E-2</v>
+        <v>0.11978340919460501</v>
       </c>
       <c r="F28" s="1">
-        <v>-0.24966019724865701</v>
+        <v>-0.18881236980518301</v>
       </c>
       <c r="G28" s="1">
-        <v>-6.7313377882591105E-2</v>
+        <v>0.280738594237669</v>
       </c>
       <c r="H28" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
@@ -3866,22 +3876,22 @@
         <v>69</v>
       </c>
       <c r="C29" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D29" s="1">
-        <v>8.1511308984761804E-2</v>
+        <v>-0.15848678756562401</v>
       </c>
       <c r="E29" s="1">
-        <v>5.1744767443281901E-2</v>
+        <v>4.6517045756649403E-2</v>
       </c>
       <c r="F29" s="1">
-        <v>-1.9908435204070801E-2</v>
+        <v>-0.24966019724865701</v>
       </c>
       <c r="G29" s="1">
-        <v>0.18293105317359401</v>
+        <v>-6.7313377882591105E-2</v>
       </c>
       <c r="H29" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
@@ -3892,22 +3902,22 @@
         <v>69</v>
       </c>
       <c r="C30" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D30" s="1">
-        <v>-0.27621797677522297</v>
+        <v>8.1511308984761804E-2</v>
       </c>
       <c r="E30" s="1">
-        <v>0.120902056867928</v>
+        <v>5.1744767443281901E-2</v>
       </c>
       <c r="F30" s="1">
-        <v>-0.51318600823636196</v>
+        <v>-1.9908435204070801E-2</v>
       </c>
       <c r="G30" s="1">
-        <v>-3.92499453140834E-2</v>
+        <v>0.18293105317359401</v>
       </c>
       <c r="H30" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
@@ -3918,19 +3928,19 @@
         <v>69</v>
       </c>
       <c r="C31" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D31" s="1">
-        <v>-0.136961627876207</v>
+        <v>-0.27621797677522297</v>
       </c>
       <c r="E31" s="1">
-        <v>5.6257626387067702E-2</v>
+        <v>0.120902056867928</v>
       </c>
       <c r="F31" s="1">
-        <v>-0.24722657559486</v>
+        <v>-0.51318600823636196</v>
       </c>
       <c r="G31" s="1">
-        <v>-2.66966801575543E-2</v>
+        <v>-3.92499453140834E-2</v>
       </c>
       <c r="H31" t="s">
         <v>127</v>
@@ -3944,22 +3954,22 @@
         <v>69</v>
       </c>
       <c r="C32" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D32" s="1">
-        <v>4.5963112216243399E-2</v>
+        <v>-0.136961627876207</v>
       </c>
       <c r="E32" s="1">
-        <v>0.11978340919460501</v>
+        <v>5.6257626387067702E-2</v>
       </c>
       <c r="F32" s="1">
-        <v>-0.18881236980518301</v>
+        <v>-0.24722657559486</v>
       </c>
       <c r="G32" s="1">
-        <v>0.280738594237669</v>
+        <v>-2.66966801575543E-2</v>
       </c>
       <c r="H32" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
@@ -3970,22 +3980,22 @@
         <v>69</v>
       </c>
       <c r="C33" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D33" s="1">
-        <v>-0.37242136583725299</v>
+        <v>-0.113076295722571</v>
       </c>
       <c r="E33" s="1">
-        <v>0.12943191505467999</v>
+        <v>0.14693490990371899</v>
       </c>
       <c r="F33" s="1">
-        <v>-0.626107919344426</v>
+        <v>-0.401068719133862</v>
       </c>
       <c r="G33" s="1">
-        <v>-0.118734812330081</v>
+        <v>0.174916127688719</v>
       </c>
       <c r="H33" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -3996,22 +4006,22 @@
         <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D34" s="1">
-        <v>-0.113076295722571</v>
+        <v>-0.37242136583725299</v>
       </c>
       <c r="E34" s="1">
-        <v>0.14693490990371899</v>
+        <v>0.12943191505467999</v>
       </c>
       <c r="F34" s="1">
-        <v>-0.401068719133862</v>
+        <v>-0.626107919344426</v>
       </c>
       <c r="G34" s="1">
-        <v>0.174916127688719</v>
+        <v>-0.118734812330081</v>
       </c>
       <c r="H34" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -4074,22 +4084,22 @@
         <v>116</v>
       </c>
       <c r="C37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D37" s="1">
-        <v>-0.12229520106668899</v>
+        <v>8.1964706406369298E-3</v>
       </c>
       <c r="E37" s="1">
-        <v>4.8582253582473603E-2</v>
+        <v>0.124959087074511</v>
       </c>
       <c r="F37" s="1">
-        <v>-0.21751641808833799</v>
+        <v>-0.23672334002540599</v>
       </c>
       <c r="G37" s="1">
-        <v>-2.7073984045041299E-2</v>
+        <v>0.25311628130667901</v>
       </c>
       <c r="H37" t="s">
-        <v>127</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
@@ -4100,22 +4110,22 @@
         <v>116</v>
       </c>
       <c r="C38" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D38" s="1">
-        <v>8.1964706406369298E-3</v>
+        <v>-0.12229520106668899</v>
       </c>
       <c r="E38" s="1">
-        <v>0.124959087074511</v>
+        <v>4.8582253582473603E-2</v>
       </c>
       <c r="F38" s="1">
-        <v>-0.23672334002540599</v>
+        <v>-0.21751641808833799</v>
       </c>
       <c r="G38" s="1">
-        <v>0.25311628130667901</v>
+        <v>-2.7073984045041299E-2</v>
       </c>
       <c r="H38" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>